<commit_message>
EPBDS-16838 Fix like skipping the pattern for an empty text and matching @ to A–Z only, textSplit resuming its search past a partial separator match, and toDate ignoring the text after the date
</commit_message>
<xml_diff>
--- a/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/7-Functions/DateFunctions.xlsx
+++ b/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/7-Functions/DateFunctions.xlsx
@@ -1316,7 +1316,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:I60"/>
+  <dimension ref="A2:I72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -1658,10 +1658,10 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="30" customHeight="1">
+    <row r="31" ht="57" customHeight="1">
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>toDate(text) reads the ISO form yyyy-MM-dd or the US form MM/dd/yyyy, with or without leading zeros. toDate(text, pattern) reads the text by a SimpleDateFormat pattern; the parts missing in the pattern are taken from January 1, 1970. A text that is not a date, a day that does not exist and a wrong pattern give an empty date.</t>
+          <t>toDate(text) reads the ISO form yyyy-MM-dd or the US form MM/dd/yyyy, with or without leading zeros. toDate(text, pattern) reads the text by a SimpleDateFormat pattern, and an empty pattern reads the forms of toDate(text); the parts missing in the pattern are taken from January 1, 1970. The whole text must be the date, while blanks around it are ignored, so a time after the date needs a pattern that reads it. A text that is not a date, more text after the date, a day that does not exist and a wrong pattern give an empty date.</t>
         </is>
       </c>
     </row>
@@ -1724,314 +1724,475 @@
     <row r="38">
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>FromPattern</t>
+          <t>FromTextWithBlanks</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>= toString(toDate("15.03.2024", "dd.MM.yyyy"))</t>
+          <t>= toString(toDate(" 2024-03-15 "))</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>FromMonthName</t>
+          <t>FromPattern</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>= toString(toDate("12-Jul-1980", "dd-MMM-yyyy"))</t>
+          <t>= toString(toDate("15.03.2024", "dd.MM.yyyy"))</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>FromQuoted</t>
+          <t>FromEmptyPattern</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>= toString(toDate("30 of 04 2015", "dd 'of' MM yyyy"))</t>
+          <t>= toString(toDate("2024-03-15", ""))</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>OnlyYear</t>
+          <t>FromDateAndTime</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>= toString(toDate("1789", "yyyy"))</t>
+          <t>= hourOfDay(toDate("2024-03-15T10:20", "yyyy-MM-dd'T'HH:mm"))</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>OnlyDay</t>
+          <t>FromMonthName</t>
         </is>
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>= toString(toDate("31", "dd"))</t>
+          <t>= toString(toDate("12-Jul-1980", "dd-MMM-yyyy"))</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>NotADate</t>
+          <t>FromQuoted</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>= toDate("abc")</t>
+          <t>= toString(toDate("30 of 04 2015", "dd 'of' MM yyyy"))</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>NoSuchDay</t>
+          <t>OnlyYear</t>
         </is>
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>= toDate("02/30/2024")</t>
+          <t>= toString(toDate("1789", "yyyy"))</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>NoSuchMonth</t>
+          <t>OnlyDay</t>
         </is>
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>= toDate("13/13/2018", "dd/MM/yyyy")</t>
+          <t>= toString(toDate("31", "dd"))</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="B46" s="6" t="inlineStr">
         <is>
+          <t>NotADate</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>= toDate("abc")</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="6" t="inlineStr">
+        <is>
+          <t>TextAfterDate</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>= toDate("04/30/2015abc")</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>TextAfterPattern</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>= toDate("15.03.2024x", "dd.MM.yyyy")</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>TimeAfterDate</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
+          <t>= toDate("2024-03-15T10:20")</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>NoSuchDay</t>
+        </is>
+      </c>
+      <c r="C50" s="7" t="inlineStr">
+        <is>
+          <t>= toDate("02/30/2024")</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>NoSuchMonth</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="inlineStr">
+        <is>
+          <t>= toDate("13/13/2018", "dd/MM/yyyy")</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="6" t="inlineStr">
+        <is>
           <t>WrongPattern</t>
         </is>
       </c>
-      <c r="C46" s="7" t="inlineStr">
+      <c r="C52" s="7" t="inlineStr">
         <is>
           <t>= toDate("12/12/2018", "as")</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="B48" s="3" t="inlineStr">
+    <row r="53"/>
+    <row r="54">
+      <c r="B54" s="3" t="inlineStr">
         <is>
           <t>Test TextToDates TextToDatesTest</t>
         </is>
       </c>
-      <c r="C48" s="8" t="n"/>
-      <c r="D48" s="4" t="n"/>
-    </row>
-    <row r="49">
-      <c r="B49" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$FromText</t>
-        </is>
-      </c>
-      <c r="C49" s="5" t="inlineStr">
-        <is>
-          <t>toString(toDate("2024-03-15"))</t>
-        </is>
-      </c>
-      <c r="D49" s="10" t="inlineStr">
-        <is>
-          <t>03/15/2024</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="B50" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$FromUsText</t>
-        </is>
-      </c>
-      <c r="C50" s="5" t="inlineStr">
-        <is>
-          <t>toString(toDate("3/5/2024"))</t>
-        </is>
-      </c>
-      <c r="D50" s="10" t="inlineStr">
-        <is>
-          <t>03/05/2024</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="B51" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$FromShortIso</t>
-        </is>
-      </c>
-      <c r="C51" s="5" t="inlineStr">
-        <is>
-          <t>toString(toDate("2024-3-5"))</t>
-        </is>
-      </c>
-      <c r="D51" s="10" t="inlineStr">
-        <is>
-          <t>03/05/2024</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="B52" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$FromPattern</t>
-        </is>
-      </c>
-      <c r="C52" s="5" t="inlineStr">
-        <is>
-          <t>toString(toDate("15.03.2024", "dd.MM.yyyy"))</t>
-        </is>
-      </c>
-      <c r="D52" s="10" t="inlineStr">
-        <is>
-          <t>03/15/2024</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="B53" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$FromMonthName</t>
-        </is>
-      </c>
-      <c r="C53" s="5" t="inlineStr">
-        <is>
-          <t>toString(toDate("12-Jul-1980", "dd-MMM-yyyy"))</t>
-        </is>
-      </c>
-      <c r="D53" s="10" t="inlineStr">
-        <is>
-          <t>07/12/1980</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="B54" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$FromQuoted</t>
-        </is>
-      </c>
-      <c r="C54" s="5" t="inlineStr">
-        <is>
-          <t>toString(toDate("30 of 04 2015", "dd 'of' MM yyyy"))</t>
-        </is>
-      </c>
-      <c r="D54" s="10" t="inlineStr">
-        <is>
-          <t>04/30/2015</t>
-        </is>
-      </c>
+      <c r="C54" s="8" t="n"/>
+      <c r="D54" s="4" t="n"/>
     </row>
     <row r="55">
       <c r="B55" s="9" t="inlineStr">
         <is>
-          <t>_res_.$OnlyYear</t>
+          <t>_res_.$FromText</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>toString(toDate("1789", "yyyy"))</t>
+          <t>toString(toDate("2024-03-15"))</t>
         </is>
       </c>
       <c r="D55" s="10" t="inlineStr">
         <is>
-          <t>01/01/1789</t>
+          <t>03/15/2024</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="B56" s="9" t="inlineStr">
         <is>
-          <t>_res_.$OnlyDay</t>
+          <t>_res_.$FromUsText</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>toString(toDate("31", "dd"))</t>
+          <t>toString(toDate("3/5/2024"))</t>
         </is>
       </c>
       <c r="D56" s="10" t="inlineStr">
         <is>
-          <t>01/31/1970</t>
+          <t>03/05/2024</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="B57" s="9" t="inlineStr">
         <is>
-          <t>_res_.$NotADate</t>
+          <t>_res_.$FromShortIso</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>toDate("abc")</t>
-        </is>
-      </c>
-      <c r="D57" s="10" t="n"/>
+          <t>toString(toDate("2024-3-5"))</t>
+        </is>
+      </c>
+      <c r="D57" s="10" t="inlineStr">
+        <is>
+          <t>03/05/2024</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="B58" s="9" t="inlineStr">
         <is>
-          <t>_res_.$NoSuchDay</t>
+          <t>_res_.$FromTextWithBlanks</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>toDate("02/30/2024")</t>
-        </is>
-      </c>
-      <c r="D58" s="10" t="n"/>
+          <t>toString(toDate(" 2024-03-15 "))</t>
+        </is>
+      </c>
+      <c r="D58" s="10" t="inlineStr">
+        <is>
+          <t>03/15/2024</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="B59" s="9" t="inlineStr">
         <is>
-          <t>_res_.$NoSuchMonth</t>
+          <t>_res_.$FromPattern</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>toDate("13/13/2018", "dd/MM/yyyy")</t>
-        </is>
-      </c>
-      <c r="D59" s="10" t="n"/>
+          <t>toString(toDate("15.03.2024", "dd.MM.yyyy"))</t>
+        </is>
+      </c>
+      <c r="D59" s="10" t="inlineStr">
+        <is>
+          <t>03/15/2024</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="B60" s="9" t="inlineStr">
         <is>
+          <t>_res_.$FromEmptyPattern</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>toString(toDate("2024-03-15", ""))</t>
+        </is>
+      </c>
+      <c r="D60" s="10" t="inlineStr">
+        <is>
+          <t>03/15/2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$FromDateAndTime</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>hourOfDay(toDate("2024-03-15T10:20", "yyyy-MM-dd'T'HH:mm"))</t>
+        </is>
+      </c>
+      <c r="D61" s="10" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$FromMonthName</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>toString(toDate("12-Jul-1980", "dd-MMM-yyyy"))</t>
+        </is>
+      </c>
+      <c r="D62" s="10" t="inlineStr">
+        <is>
+          <t>07/12/1980</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$FromQuoted</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>toString(toDate("30 of 04 2015", "dd 'of' MM yyyy"))</t>
+        </is>
+      </c>
+      <c r="D63" s="10" t="inlineStr">
+        <is>
+          <t>04/30/2015</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$OnlyYear</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="inlineStr">
+        <is>
+          <t>toString(toDate("1789", "yyyy"))</t>
+        </is>
+      </c>
+      <c r="D64" s="10" t="inlineStr">
+        <is>
+          <t>01/01/1789</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$OnlyDay</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>toString(toDate("31", "dd"))</t>
+        </is>
+      </c>
+      <c r="D65" s="10" t="inlineStr">
+        <is>
+          <t>01/31/1970</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$NotADate</t>
+        </is>
+      </c>
+      <c r="C66" s="5" t="inlineStr">
+        <is>
+          <t>toDate("abc")</t>
+        </is>
+      </c>
+      <c r="D66" s="10" t="n"/>
+    </row>
+    <row r="67">
+      <c r="B67" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$TextAfterDate</t>
+        </is>
+      </c>
+      <c r="C67" s="5" t="inlineStr">
+        <is>
+          <t>toDate("04/30/2015abc")</t>
+        </is>
+      </c>
+      <c r="D67" s="10" t="n"/>
+    </row>
+    <row r="68">
+      <c r="B68" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$TextAfterPattern</t>
+        </is>
+      </c>
+      <c r="C68" s="5" t="inlineStr">
+        <is>
+          <t>toDate("15.03.2024x", "dd.MM.yyyy")</t>
+        </is>
+      </c>
+      <c r="D68" s="10" t="n"/>
+    </row>
+    <row r="69">
+      <c r="B69" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$TimeAfterDate</t>
+        </is>
+      </c>
+      <c r="C69" s="5" t="inlineStr">
+        <is>
+          <t>toDate("2024-03-15T10:20")</t>
+        </is>
+      </c>
+      <c r="D69" s="10" t="n"/>
+    </row>
+    <row r="70">
+      <c r="B70" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$NoSuchDay</t>
+        </is>
+      </c>
+      <c r="C70" s="5" t="inlineStr">
+        <is>
+          <t>toDate("02/30/2024")</t>
+        </is>
+      </c>
+      <c r="D70" s="10" t="n"/>
+    </row>
+    <row r="71">
+      <c r="B71" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$NoSuchMonth</t>
+        </is>
+      </c>
+      <c r="C71" s="5" t="inlineStr">
+        <is>
+          <t>toDate("13/13/2018", "dd/MM/yyyy")</t>
+        </is>
+      </c>
+      <c r="D71" s="10" t="n"/>
+    </row>
+    <row r="72">
+      <c r="B72" s="9" t="inlineStr">
+        <is>
           <t>_res_.$WrongPattern</t>
         </is>
       </c>
-      <c r="C60" s="5" t="inlineStr">
+      <c r="C72" s="5" t="inlineStr">
         <is>
           <t>toDate("12/12/2018", "as")</t>
         </is>
       </c>
-      <c r="D60" s="10" t="n"/>
+      <c r="D72" s="10" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B19:D19"/>
+    <mergeCell ref="B54:D54"/>
     <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B48:D48"/>
     <mergeCell ref="B31:I31"/>
     <mergeCell ref="B4:I4"/>
   </mergeCells>

</xml_diff>